<commit_message>
Add test.step and new test cases: logout, empty fields, cart persistence
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -729,35 +729,151 @@
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>TC_LOGIN_04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Log out returns the nav to its logged-out state</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>1. Click Log out</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Log in link reappears; Welcome &lt;username&gt; and Log out are hidden</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>tests/ui/login.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Login with both fields empty</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>1. Click Log in
+2. Leave Username and Password empty
+3. Submit</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Alert "Please fill out Username and Password." is shown</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>tests/ui/login.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="62" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>TC_CART_01</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Cart</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Add a product to cart while logged in, then place an order</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>1. Open a product from Home
 2. Click Add to cart, accept the confirmation
@@ -766,59 +882,59 @@
 5. Confirm the purchase</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Purchase confirmation modal appears; after closing it, Home loads and the cart is empty</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>tests/ui/purchaseOrder.spec.ts</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="62" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8" ht="62" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>TC_CART_02</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Cart</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Add multiple products to cart as a guest, then delete one</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>User is NOT logged in</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>1. From Home, add the 1st product to cart
 2. Add the 2nd product to cart
@@ -826,200 +942,258 @@
 4. Delete the 1st product</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Cart shows both products added; after deleting one, only the other product remains</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>tests/ui/cart.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="62" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TC_API_01</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Product Catalog</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>GET /entries returns the product catalog</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>1. Send GET /entries</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Status 200, Items non-empty, a known product's fields match, body matches schema</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>tests/api/getAllProducts.spec.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TC_API_02</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Product Catalog</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>POST /view returns a single product by id</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Product id 1 exists</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>1. Send POST /view with { id: "1" }</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Status 200, returned fields match the known product, body matches schema</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>tests/api/getProductById.spec.ts</t>
         </is>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>TC_CART_03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Cart contents persist after a page reload</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>User is NOT logged in, 1 product already in cart</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>1. Add a product to cart as a guest
+2. Reload the page</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>The same product is still in the cart after reload</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>tests/ui/cart.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="62" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC_API_01</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Product Catalog</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>GET /entries returns the product catalog</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>1. Send GET /entries</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Status 200, Items non-empty, a known product's fields match, body matches schema</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>tests/api/getAllProducts.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="62" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC_API_02</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Product Catalog</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>POST /view returns a single product by id</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Product id 1 exists</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>1. Send POST /view with { id: "1" }</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Status 200, returned fields match the known product, body matches schema</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>tests/api/getProductById.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="62" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>TC_API_03</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Product Catalog</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>API</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>POST /view with a non-existent product id</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Product id 999999 does not exist</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>1. Send POST /view with { id: "999999" }</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Status 200, body is { errorMessage: "Not found." }</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>tests/api/getProductById.spec.ts</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Note: lists only the cases covered by the automated suite in this repo (tests/ui, tests/api). Each row's ID is prefixed in its test's title in code, and the Automated Test column names the spec file, for traceability. All rows are Automated = Yes.</t>
         </is>

</xml_diff>